<commit_message>
Add disguised push notifications for offline messages
</commit_message>
<xml_diff>
--- a/New Microsoft Excel Worksheet.xlsx
+++ b/New Microsoft Excel Worksheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\todo-app\Auralook\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3294F643-CC82-49A2-9735-1A3B0F73D2BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E767BCF-EBC6-42C2-B924-4297BAEF2629}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="23280" windowHeight="14880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="14">
   <si>
     <t xml:space="preserve">url </t>
   </si>
@@ -55,16 +55,36 @@
   </si>
   <si>
     <t>https://authentication-affq.onrender.com</t>
+  </si>
+  <si>
+    <t>https://console.cron-job.org/</t>
+  </si>
+  <si>
+    <t>For active</t>
+  </si>
+  <si>
+    <t>Cronjob@786</t>
+  </si>
+  <si>
+    <t>cronjob</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -87,13 +107,16 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -372,13 +395,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="31.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="39.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -389,7 +415,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -397,7 +423,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -405,7 +431,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -413,7 +439,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>7</v>
       </c>
@@ -421,7 +447,24 @@
         <v>6</v>
       </c>
     </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C6" t="s">
+        <v>10</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="D6" r:id="rId1" xr:uid="{EA284766-2BCD-4B28-A67B-329039843043}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>